<commit_message>
Cập nhật công cụ xử lý hồ sơ và GCN
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python\DAYHSQUET\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E7FA10E-BA39-45EC-80D1-38AE6CD6828A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6584CF01-3BEA-40D2-87F2-C33320FA9D80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -361,10 +361,10 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B2">
-        <v>431</v>
+        <v>280</v>
       </c>
     </row>
   </sheetData>

</xml_diff>